<commit_message>
Update honors pacing guide + fix review-day chapter detection
- grade_6_advanced.xlsx: review/test days now use PDF filename as lesson
  (e.g. "6_1_test") for explicit bank routing
- pacing.py: review_chapter detection now matches "6_N_test" / "6_N_mc"
  filename patterns in addition to free-text "Ch N Review" patterns

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pacing_guides/grade_6_advanced.xlsx
+++ b/pacing_guides/grade_6_advanced.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="291">
   <si>
     <t>Lesson</t>
   </si>
@@ -128,13 +128,16 @@
     <t>Labor Day - NO SCHOOL</t>
   </si>
   <si>
-    <t>Review Day</t>
+    <t>6_1_test</t>
+  </si>
+  <si>
+    <t>Chapter 1 Review</t>
   </si>
   <si>
     <t>Day 10</t>
   </si>
   <si>
-    <t>Test Day Ch 1</t>
+    <t>Chapter 1 Test</t>
   </si>
   <si>
     <t>Day 11</t>
@@ -200,96 +203,111 @@
     <t>Day 20</t>
   </si>
   <si>
+    <t>6_2_mc</t>
+  </si>
+  <si>
+    <t>Chapter 2 Review</t>
+  </si>
+  <si>
+    <t>Day 21</t>
+  </si>
+  <si>
+    <t>Half Day</t>
+  </si>
+  <si>
+    <t>6_2_test</t>
+  </si>
+  <si>
+    <t>Day 22</t>
+  </si>
+  <si>
+    <t>Test Chapter 2</t>
+  </si>
+  <si>
+    <t>Integers</t>
+  </si>
+  <si>
+    <t>Day 23</t>
+  </si>
+  <si>
+    <t>Compare and Order Integers</t>
+  </si>
+  <si>
+    <t>Day 24</t>
+  </si>
+  <si>
+    <t>Rational Numbers</t>
+  </si>
+  <si>
+    <t>Day 25</t>
+  </si>
+  <si>
+    <t>Absolute Value</t>
+  </si>
+  <si>
+    <t>Day 26</t>
+  </si>
+  <si>
+    <t>Coordinate Plane</t>
+  </si>
+  <si>
+    <t>Day 27</t>
+  </si>
+  <si>
+    <t>Polygons in the Coordinate Plane</t>
+  </si>
+  <si>
+    <t>Day 28</t>
+  </si>
+  <si>
+    <t>6_3_test</t>
+  </si>
+  <si>
+    <t>Day 29</t>
+  </si>
+  <si>
+    <t>Day 30</t>
+  </si>
+  <si>
+    <t>Test Chapter 3</t>
+  </si>
+  <si>
+    <t>Adding integers</t>
+  </si>
+  <si>
+    <t>Day 31</t>
+  </si>
+  <si>
+    <t>Adding rational numbers</t>
+  </si>
+  <si>
+    <t>Day 32</t>
+  </si>
+  <si>
+    <t>Day 33</t>
+  </si>
+  <si>
+    <t>Subtracting Integers</t>
+  </si>
+  <si>
+    <t>Day 34</t>
+  </si>
+  <si>
+    <t>F/END Q1</t>
+  </si>
+  <si>
+    <t>Subtracting Rational numbers</t>
+  </si>
+  <si>
+    <t>Day 35</t>
+  </si>
+  <si>
+    <t>6_4_test</t>
+  </si>
+  <si>
     <t>Review</t>
   </si>
   <si>
-    <t>Day 21</t>
-  </si>
-  <si>
-    <t>Half Day</t>
-  </si>
-  <si>
-    <t>Day 22</t>
-  </si>
-  <si>
-    <t>Test Chapter 2</t>
-  </si>
-  <si>
-    <t>Integers</t>
-  </si>
-  <si>
-    <t>Day 23</t>
-  </si>
-  <si>
-    <t>Compare and Order Integers</t>
-  </si>
-  <si>
-    <t>Day 24</t>
-  </si>
-  <si>
-    <t>Rational Numbers</t>
-  </si>
-  <si>
-    <t>Day 25</t>
-  </si>
-  <si>
-    <t>Absolute Value</t>
-  </si>
-  <si>
-    <t>Day 26</t>
-  </si>
-  <si>
-    <t>Coordinate Plane</t>
-  </si>
-  <si>
-    <t>Day 27</t>
-  </si>
-  <si>
-    <t>Polygons in the Coordinate Plane</t>
-  </si>
-  <si>
-    <t>Day 28</t>
-  </si>
-  <si>
-    <t>Day 29</t>
-  </si>
-  <si>
-    <t>Day 30</t>
-  </si>
-  <si>
-    <t>Test Chapter 3</t>
-  </si>
-  <si>
-    <t>Adding integers</t>
-  </si>
-  <si>
-    <t>Day 31</t>
-  </si>
-  <si>
-    <t>Adding rational numbers</t>
-  </si>
-  <si>
-    <t>Day 32</t>
-  </si>
-  <si>
-    <t>Day 33</t>
-  </si>
-  <si>
-    <t>Subtracting Integers</t>
-  </si>
-  <si>
-    <t>Day 34</t>
-  </si>
-  <si>
-    <t>F/END Q1</t>
-  </si>
-  <si>
-    <t>Subtracting Rational numbers</t>
-  </si>
-  <si>
-    <t>Day 35</t>
-  </si>
-  <si>
     <t>Day 36</t>
   </si>
   <si>
@@ -518,108 +536,210 @@
     <t>Rates/unit rates</t>
   </si>
   <si>
+    <t>Day 72</t>
+  </si>
+  <si>
     <t>converting measures</t>
   </si>
   <si>
+    <t>Day 73</t>
+  </si>
+  <si>
     <t>Ratio problem solving</t>
   </si>
   <si>
+    <t>Day 74</t>
+  </si>
+  <si>
+    <t>Day 75</t>
+  </si>
+  <si>
     <t>Chapter 8 Test</t>
   </si>
   <si>
     <t>Percents and fractions</t>
   </si>
   <si>
+    <t>Day 76</t>
+  </si>
+  <si>
     <t>Percents and decimals</t>
   </si>
   <si>
+    <t>Day 77</t>
+  </si>
+  <si>
     <t>Benchmark percents</t>
   </si>
   <si>
+    <t>Day 78</t>
+  </si>
+  <si>
+    <t>Day 79</t>
+  </si>
+  <si>
     <t>Compare and order fractions, decimals, percents</t>
   </si>
   <si>
+    <t>Day 80</t>
+  </si>
+  <si>
     <t>Percent proportion</t>
   </si>
   <si>
+    <t>Day 81</t>
+  </si>
+  <si>
     <t>Percent equation</t>
   </si>
   <si>
+    <t>Day 82</t>
+  </si>
+  <si>
     <t>Percent review/PS</t>
   </si>
   <si>
+    <t>Day 83</t>
+  </si>
+  <si>
     <t>Presidents' Day - NO SCHOOL</t>
   </si>
   <si>
     <t>Percent increase/decrease</t>
   </si>
   <si>
+    <t>Day 85</t>
+  </si>
+  <si>
     <t>Discounts/markup</t>
   </si>
   <si>
+    <t>Day 86</t>
+  </si>
+  <si>
     <t>Simple Interest</t>
   </si>
   <si>
     <t>Simple interest</t>
   </si>
   <si>
+    <t>Day 87</t>
+  </si>
+  <si>
+    <t>Day 88</t>
+  </si>
+  <si>
+    <t>Day 89</t>
+  </si>
+  <si>
     <t>Chapter 9 Test</t>
   </si>
   <si>
+    <t>Day 90</t>
+  </si>
+  <si>
     <t>Area review - rectangles, squares</t>
   </si>
   <si>
     <t>Area of parallelograms</t>
   </si>
   <si>
+    <t>Day 91</t>
+  </si>
+  <si>
     <t>base and height of triangles</t>
   </si>
   <si>
+    <t>Day 92</t>
+  </si>
+  <si>
     <t>Area of triangles</t>
   </si>
   <si>
+    <t>Day 93</t>
+  </si>
+  <si>
     <t>Half Day / Open House</t>
   </si>
   <si>
     <t>area of trapezoids</t>
   </si>
   <si>
+    <t>Day 94</t>
+  </si>
+  <si>
     <t>area review and problem solving</t>
   </si>
   <si>
     <t>Three-dimensional figures</t>
   </si>
   <si>
+    <t>Day 95</t>
+  </si>
+  <si>
     <t>Surface area of prisms</t>
   </si>
   <si>
+    <t>Day 96</t>
+  </si>
+  <si>
     <t>Surface area of pyramids</t>
   </si>
   <si>
+    <t>Day 97</t>
+  </si>
+  <si>
     <t>Nets</t>
   </si>
   <si>
+    <t>Day 98</t>
+  </si>
+  <si>
     <t>Volume of rectangular prisms</t>
   </si>
   <si>
+    <t>Day 99</t>
+  </si>
+  <si>
+    <t>Day 100</t>
+  </si>
+  <si>
     <t>Chapter 10 Test</t>
   </si>
   <si>
+    <t>Day 101</t>
+  </si>
+  <si>
     <t>Circles warmup/constructions</t>
   </si>
   <si>
+    <t>Day 102</t>
+  </si>
+  <si>
     <t>Circles and circumference</t>
   </si>
   <si>
+    <t>Day 103</t>
+  </si>
+  <si>
     <t>Area of circles</t>
   </si>
   <si>
+    <t>Day 104</t>
+  </si>
+  <si>
     <t>Circles problem solving</t>
   </si>
   <si>
+    <t>Day 105</t>
+  </si>
+  <si>
     <t>Th/END Q3</t>
   </si>
   <si>
+    <t>Day 106</t>
+  </si>
+  <si>
     <t>3/26 - 4/2</t>
   </si>
   <si>
@@ -632,30 +752,66 @@
     <t>Perimeters and areas of composite figures</t>
   </si>
   <si>
+    <t>Day 107</t>
+  </si>
+  <si>
     <t>Constructing polygons</t>
   </si>
   <si>
+    <t>Day 108</t>
+  </si>
+  <si>
     <t>constructions</t>
   </si>
   <si>
+    <t>Day 109</t>
+  </si>
+  <si>
     <t>constuctions</t>
   </si>
   <si>
+    <t>Day 110</t>
+  </si>
+  <si>
     <t>Finding unknown angle measures</t>
   </si>
   <si>
+    <t>Day 111</t>
+  </si>
+  <si>
+    <t>Day 112</t>
+  </si>
+  <si>
+    <t>Day 113</t>
+  </si>
+  <si>
+    <t>Day 114</t>
+  </si>
+  <si>
     <t>Chapter 11 Test</t>
   </si>
   <si>
     <t>Statistical questions</t>
   </si>
   <si>
+    <t>Day 115</t>
+  </si>
+  <si>
     <t>Mean</t>
   </si>
   <si>
+    <t>Day 116</t>
+  </si>
+  <si>
+    <t>Day 117</t>
+  </si>
+  <si>
     <t>Measures of Center</t>
   </si>
   <si>
+    <t>Day 118</t>
+  </si>
+  <si>
     <t>Meaures of variation</t>
   </si>
   <si>
@@ -668,28 +824,64 @@
     <t>Measures of variation</t>
   </si>
   <si>
+    <t>Day 119</t>
+  </si>
+  <si>
     <t>MAD</t>
   </si>
   <si>
+    <t>Day 120</t>
+  </si>
+  <si>
     <t>Stem-and-leaf plots</t>
   </si>
   <si>
+    <t>Day 121</t>
+  </si>
+  <si>
     <t>Histograms</t>
   </si>
   <si>
+    <t>Day 122</t>
+  </si>
+  <si>
     <t>Shapes of distributions</t>
   </si>
   <si>
+    <t>Day 123</t>
+  </si>
+  <si>
     <t>Choosing appropriate measures</t>
   </si>
   <si>
+    <t>Day 124</t>
+  </si>
+  <si>
     <t>Box-and Wisker plots</t>
   </si>
   <si>
+    <t>Day 125</t>
+  </si>
+  <si>
     <t>Half Day / Arts Celebration</t>
   </si>
   <si>
+    <t>Day 126</t>
+  </si>
+  <si>
     <t>Chapter 12 &amp; 13 Assessment</t>
+  </si>
+  <si>
+    <t>Day 127</t>
+  </si>
+  <si>
+    <t>Day 128</t>
+  </si>
+  <si>
+    <t>Day 129</t>
+  </si>
+  <si>
+    <t>Day 130</t>
   </si>
   <si>
     <t>Memorial Day - NO SCHOOL</t>
@@ -770,10 +962,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
@@ -1291,8 +1483,11 @@
       <c r="E18" s="5" t="s">
         <v>36</v>
       </c>
+      <c r="F18" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="G18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19">
@@ -1306,10 +1501,13 @@
         <v>19</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
@@ -1323,13 +1521,13 @@
         <v>6</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="6" t="s">
         <v>41</v>
       </c>
+      <c r="F20" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="G20" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -1343,10 +1541,10 @@
         <v>9</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="6" t="s">
         <v>41</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -1360,14 +1558,14 @@
       <c r="C23" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="6">
         <v>2.2</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>43</v>
+      <c r="F23" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -1380,14 +1578,14 @@
       <c r="C24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="6">
         <v>2.2</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>43</v>
+      <c r="F24" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -1401,13 +1599,13 @@
         <v>19</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F25" s="6" t="s">
         <v>47</v>
       </c>
+      <c r="F25" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="G25" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -1420,14 +1618,14 @@
       <c r="C26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="6">
         <v>2.3</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>47</v>
+      <c r="F26" s="5" t="s">
+        <v>48</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -1443,8 +1641,8 @@
       <c r="E27" s="4">
         <v>2.4</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>50</v>
+      <c r="F27" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
@@ -1458,14 +1656,14 @@
       <c r="C29" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="6">
         <v>2.5</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>51</v>
+      <c r="F29" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
@@ -1478,14 +1676,14 @@
       <c r="C30" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="6">
         <v>2.6</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>53</v>
+      <c r="F30" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -1496,7 +1694,7 @@
         <v>19</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -1509,14 +1707,14 @@
       <c r="C32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="6">
         <v>2.7</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>56</v>
+      <c r="F32" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
@@ -1532,8 +1730,8 @@
       <c r="E33" s="4">
         <v>2.8</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>58</v>
+      <c r="F33" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1"/>
@@ -1547,14 +1745,14 @@
       <c r="C35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="6">
         <v>2.8</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>58</v>
+      <c r="F35" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
@@ -1567,12 +1765,14 @@
       <c r="C36" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="6" t="s">
-        <v>60</v>
+      <c r="E36" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>62</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
@@ -1583,7 +1783,7 @@
         <v>19</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -1597,14 +1797,16 @@
         <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F38" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E38" s="1"/>
-      <c r="F38" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="G38" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -1618,8 +1820,8 @@
         <v>9</v>
       </c>
       <c r="E39" s="1"/>
-      <c r="F39" s="6" t="s">
-        <v>64</v>
+      <c r="F39" s="5" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1"/>
@@ -1636,11 +1838,11 @@
       <c r="E41" s="4">
         <v>3.1</v>
       </c>
-      <c r="F41" s="6" t="s">
-        <v>65</v>
+      <c r="F41" s="5" t="s">
+        <v>68</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
@@ -1656,11 +1858,11 @@
       <c r="E42" s="4">
         <v>3.2</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>67</v>
+      <c r="F42" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -1676,11 +1878,11 @@
       <c r="E43" s="4">
         <v>3.3</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>69</v>
+      <c r="F43" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -1696,11 +1898,11 @@
       <c r="E44" s="4">
         <v>3.4</v>
       </c>
-      <c r="F44" s="6" t="s">
-        <v>71</v>
+      <c r="F44" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -1716,8 +1918,8 @@
       <c r="E45" s="4">
         <v>3.5</v>
       </c>
-      <c r="F45" s="6" t="s">
-        <v>73</v>
+      <c r="F45" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1"/>
@@ -1731,14 +1933,14 @@
       <c r="C47" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E47" s="5">
+      <c r="E47" s="6">
         <v>3.5</v>
       </c>
-      <c r="F47" s="6" t="s">
-        <v>73</v>
+      <c r="F47" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -1751,14 +1953,14 @@
       <c r="C48" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E48" s="5">
+      <c r="E48" s="6">
         <v>3.6</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>75</v>
+      <c r="F48" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -1772,10 +1974,10 @@
         <v>19</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -1789,10 +1991,10 @@
         <v>6</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -1806,8 +2008,8 @@
         <v>9</v>
       </c>
       <c r="E51" s="1"/>
-      <c r="F51" s="6" t="s">
-        <v>79</v>
+      <c r="F51" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -1824,11 +2026,11 @@
       <c r="E53" s="4">
         <v>4.1</v>
       </c>
-      <c r="F53" s="6" t="s">
-        <v>80</v>
+      <c r="F53" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
@@ -1844,11 +2046,11 @@
       <c r="E54" s="4">
         <v>4.2</v>
       </c>
-      <c r="F54" s="6" t="s">
-        <v>82</v>
+      <c r="F54" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
@@ -1864,11 +2066,11 @@
       <c r="E55" s="4">
         <v>4.2</v>
       </c>
-      <c r="F55" s="6" t="s">
-        <v>82</v>
+      <c r="F55" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
@@ -1884,11 +2086,11 @@
       <c r="E56" s="4">
         <v>4.3</v>
       </c>
-      <c r="F56" s="6" t="s">
-        <v>85</v>
+      <c r="F56" s="5" t="s">
+        <v>89</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -1899,14 +2101,14 @@
         <v>46318.0</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D57" s="7"/>
       <c r="E57" s="4">
         <v>4.3</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G57" s="7"/>
       <c r="H57" s="10"/>
@@ -1924,14 +2126,14 @@
       <c r="C59" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E59" s="5">
+      <c r="E59" s="6">
         <v>4.4</v>
       </c>
-      <c r="F59" s="6" t="s">
-        <v>88</v>
+      <c r="F59" s="5" t="s">
+        <v>92</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -1944,12 +2146,14 @@
       <c r="C60" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E60" s="1"/>
-      <c r="F60" s="6" t="s">
-        <v>60</v>
+      <c r="E60" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -1963,11 +2167,11 @@
         <v>19</v>
       </c>
       <c r="E61" s="1"/>
-      <c r="F61" s="6" t="s">
-        <v>91</v>
+      <c r="F61" s="5" t="s">
+        <v>97</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -1978,7 +2182,7 @@
         <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E62" s="1"/>
     </row>
@@ -1990,7 +2194,7 @@
         <v>9</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E63" s="1"/>
     </row>
@@ -2005,14 +2209,14 @@
       <c r="C65" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E65" s="5">
+      <c r="E65" s="6">
         <v>5.1</v>
       </c>
-      <c r="F65" s="6" t="s">
-        <v>94</v>
+      <c r="F65" s="5" t="s">
+        <v>100</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
@@ -2025,14 +2229,14 @@
       <c r="C66" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E66" s="5">
+      <c r="E66" s="6">
         <v>5.2</v>
       </c>
-      <c r="F66" s="6" t="s">
-        <v>96</v>
+      <c r="F66" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
@@ -2048,11 +2252,11 @@
       <c r="E67" s="4">
         <v>5.3</v>
       </c>
-      <c r="F67" s="6" t="s">
-        <v>98</v>
+      <c r="F67" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="J67" s="1"/>
     </row>
@@ -2067,16 +2271,16 @@
         <v>6</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E68" s="4">
         <v>5.4</v>
       </c>
-      <c r="F68" s="6" t="s">
-        <v>100</v>
+      <c r="F68" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="J68" s="1"/>
     </row>
@@ -2093,8 +2297,8 @@
       <c r="E69" s="4">
         <v>5.4</v>
       </c>
-      <c r="F69" s="6" t="s">
-        <v>100</v>
+      <c r="F69" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="J69" s="1"/>
     </row>
@@ -2112,11 +2316,11 @@
       <c r="E71" s="4">
         <v>5.5</v>
       </c>
-      <c r="F71" s="6" t="s">
-        <v>102</v>
+      <c r="F71" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
@@ -2132,11 +2336,11 @@
       <c r="E72" s="4">
         <v>5.5</v>
       </c>
-      <c r="F72" s="6" t="s">
-        <v>102</v>
+      <c r="F72" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
@@ -2147,7 +2351,7 @@
         <v>19</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
@@ -2161,11 +2365,11 @@
         <v>6</v>
       </c>
       <c r="E74" s="1"/>
-      <c r="F74" s="6" t="s">
-        <v>60</v>
+      <c r="F74" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
@@ -2179,8 +2383,8 @@
         <v>9</v>
       </c>
       <c r="E75" s="3"/>
-      <c r="F75" s="6" t="s">
-        <v>107</v>
+      <c r="F75" s="5" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1"/>
@@ -2194,14 +2398,14 @@
       <c r="C77" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E77" s="5">
+      <c r="E77" s="6">
         <v>6.1</v>
       </c>
-      <c r="F77" s="6" t="s">
-        <v>108</v>
+      <c r="F77" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
@@ -2214,14 +2418,14 @@
       <c r="C78" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E78" s="5">
+      <c r="E78" s="6">
         <v>6.2</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>110</v>
+      <c r="F78" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
@@ -2234,14 +2438,14 @@
       <c r="C79" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E79" s="5">
+      <c r="E79" s="6">
         <v>6.3</v>
       </c>
-      <c r="F79" s="6" t="s">
-        <v>112</v>
+      <c r="F79" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
@@ -2254,14 +2458,14 @@
       <c r="C80" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E80" s="5">
+      <c r="E80" s="6">
         <v>6.3</v>
       </c>
-      <c r="F80" s="6" t="s">
-        <v>112</v>
+      <c r="F80" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
@@ -2275,20 +2479,20 @@
         <v>9</v>
       </c>
       <c r="E81" s="1"/>
-      <c r="F81" s="6" t="s">
-        <v>60</v>
+      <c r="F81" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1"/>
     <row r="83" ht="15.75" customHeight="1">
       <c r="B83" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1"/>
@@ -2302,14 +2506,14 @@
       <c r="C85" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E85" s="5">
+      <c r="E85" s="6">
         <v>6.4</v>
       </c>
-      <c r="F85" s="6" t="s">
-        <v>118</v>
+      <c r="F85" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
@@ -2322,14 +2526,14 @@
       <c r="C86" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E86" s="5">
+      <c r="E86" s="6">
         <v>6.4</v>
       </c>
-      <c r="F86" s="6" t="s">
-        <v>118</v>
+      <c r="F86" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
@@ -2342,14 +2546,14 @@
       <c r="C87" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E87" s="5">
+      <c r="E87" s="6">
         <v>6.5</v>
       </c>
-      <c r="F87" s="6" t="s">
-        <v>121</v>
+      <c r="F87" s="5" t="s">
+        <v>127</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
@@ -2363,14 +2567,14 @@
         <v>6</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E88" s="1"/>
-      <c r="F88" s="6" t="s">
-        <v>60</v>
+      <c r="F88" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
@@ -2384,8 +2588,8 @@
         <v>9</v>
       </c>
       <c r="E89" s="1"/>
-      <c r="F89" s="6" t="s">
-        <v>124</v>
+      <c r="F89" s="5" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1"/>
@@ -2402,11 +2606,11 @@
       <c r="E91" s="4">
         <v>7.1</v>
       </c>
-      <c r="F91" s="6" t="s">
-        <v>125</v>
+      <c r="F91" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
@@ -2422,11 +2626,11 @@
       <c r="E92" s="4">
         <v>7.2</v>
       </c>
-      <c r="F92" s="6" t="s">
-        <v>127</v>
+      <c r="F92" s="5" t="s">
+        <v>133</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
@@ -2442,11 +2646,11 @@
       <c r="E93" s="4">
         <v>7.3</v>
       </c>
-      <c r="F93" s="6" t="s">
-        <v>129</v>
+      <c r="F93" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
@@ -2460,13 +2664,13 @@
         <v>6</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="F94" s="6" t="s">
-        <v>132</v>
+        <v>137</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>138</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
@@ -2480,8 +2684,8 @@
         <v>9</v>
       </c>
       <c r="E95" s="1"/>
-      <c r="F95" s="6" t="s">
-        <v>132</v>
+      <c r="F95" s="5" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1"/>
@@ -2495,14 +2699,14 @@
       <c r="C97" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E97" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F97" s="6" t="s">
-        <v>134</v>
+      <c r="E97" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
@@ -2515,14 +2719,14 @@
       <c r="C98" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E98" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F98" s="6" t="s">
-        <v>136</v>
+      <c r="E98" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
@@ -2535,14 +2739,14 @@
       <c r="C99" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E99" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F99" s="6" t="s">
-        <v>138</v>
+      <c r="E99" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F99" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1">
@@ -2555,14 +2759,14 @@
       <c r="C100" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E100" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F100" s="6" t="s">
-        <v>138</v>
+      <c r="E100" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="G100" s="1" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
@@ -2576,19 +2780,19 @@
         <v>9</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1"/>
     <row r="103" ht="15.75" customHeight="1">
       <c r="B103" s="1" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1"/>
@@ -2602,14 +2806,14 @@
       <c r="C105" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E105" s="5">
+      <c r="E105" s="6">
         <v>7.4</v>
       </c>
-      <c r="F105" s="6" t="s">
-        <v>144</v>
+      <c r="F105" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
@@ -2622,14 +2826,14 @@
       <c r="C106" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E106" s="5">
+      <c r="E106" s="6">
         <v>7.4</v>
       </c>
-      <c r="F106" s="6" t="s">
-        <v>144</v>
+      <c r="F106" s="5" t="s">
+        <v>150</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="107" ht="15.75" customHeight="1">
@@ -2642,14 +2846,14 @@
       <c r="C107" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E107" s="5">
+      <c r="E107" s="6">
         <v>7.5</v>
       </c>
-      <c r="F107" s="6" t="s">
-        <v>147</v>
+      <c r="F107" s="5" t="s">
+        <v>153</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="108" ht="15.75" customHeight="1">
@@ -2662,11 +2866,11 @@
       <c r="C108" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F108" s="6" t="s">
-        <v>60</v>
+      <c r="F108" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="G108" s="1" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="109" ht="15.75" customHeight="1">
@@ -2679,8 +2883,8 @@
       <c r="C109" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F109" s="6" t="s">
-        <v>150</v>
+      <c r="F109" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="110" ht="15.75" customHeight="1"/>
@@ -2694,14 +2898,14 @@
       <c r="C111" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E111" s="6">
+      <c r="E111" s="5">
         <v>8.1</v>
       </c>
-      <c r="F111" s="6" t="s">
-        <v>151</v>
+      <c r="F111" s="5" t="s">
+        <v>157</v>
       </c>
       <c r="G111" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="112" ht="15.75" customHeight="1">
@@ -2714,14 +2918,14 @@
       <c r="C112" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E112" s="6">
+      <c r="E112" s="5">
         <v>8.1</v>
       </c>
-      <c r="F112" s="6" t="s">
-        <v>151</v>
+      <c r="F112" s="5" t="s">
+        <v>157</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="113" ht="15.75" customHeight="1">
@@ -2734,14 +2938,14 @@
       <c r="C113" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E113" s="5">
+      <c r="E113" s="6">
         <v>8.2</v>
       </c>
-      <c r="F113" s="6" t="s">
-        <v>154</v>
+      <c r="F113" s="5" t="s">
+        <v>160</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="114" ht="15.75" customHeight="1">
@@ -2754,14 +2958,14 @@
       <c r="C114" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E114" s="5">
+      <c r="E114" s="6">
         <v>8.3</v>
       </c>
-      <c r="F114" s="6" t="s">
-        <v>156</v>
+      <c r="F114" s="5" t="s">
+        <v>162</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
@@ -2774,11 +2978,11 @@
       <c r="C115" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E115" s="5">
+      <c r="E115" s="6">
         <v>8.3</v>
       </c>
-      <c r="F115" s="6" t="s">
-        <v>156</v>
+      <c r="F115" s="5" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="116" ht="15.75" customHeight="1"/>
@@ -2790,7 +2994,7 @@
         <v>11</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="118" ht="15.75" customHeight="1">
@@ -2803,14 +3007,14 @@
       <c r="C118" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E118" s="5">
+      <c r="E118" s="6">
         <v>8.4</v>
       </c>
-      <c r="F118" s="6" t="s">
-        <v>159</v>
+      <c r="F118" s="5" t="s">
+        <v>165</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
@@ -2823,14 +3027,14 @@
       <c r="C119" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E119" s="5">
+      <c r="E119" s="6">
         <v>8.4</v>
       </c>
-      <c r="F119" s="6" t="s">
-        <v>159</v>
+      <c r="F119" s="5" t="s">
+        <v>165</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
@@ -2843,14 +3047,14 @@
       <c r="C120" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E120" s="5">
+      <c r="E120" s="6">
         <v>8.5</v>
       </c>
-      <c r="F120" s="6" t="s">
-        <v>162</v>
+      <c r="F120" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="G120" s="1" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
@@ -2861,14 +3065,14 @@
         <v>46409.0</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D121" s="7"/>
       <c r="E121" s="11">
         <v>8.5</v>
       </c>
       <c r="F121" s="9" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G121" s="7"/>
       <c r="H121" s="10"/>
@@ -3788,14 +3992,14 @@
       <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="5">
+      <c r="E1" s="6">
         <v>8.5</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8</v>
+      <c r="F1" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="2">
@@ -3808,14 +4012,14 @@
       <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="6">
         <v>8.6</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>14</v>
+      <c r="F2" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="3">
@@ -3828,14 +4032,14 @@
       <c r="C3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>18</v>
+      <c r="E3" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="4">
@@ -3849,11 +4053,11 @@
         <v>6</v>
       </c>
       <c r="E4" s="1"/>
-      <c r="F4" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>20</v>
+      <c r="F4" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="5">
@@ -3867,8 +4071,8 @@
         <v>9</v>
       </c>
       <c r="E5" s="1"/>
-      <c r="F5" s="6" t="s">
-        <v>168</v>
+      <c r="F5" s="5" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="7">
@@ -3881,14 +4085,14 @@
       <c r="C7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="6">
         <v>9.1</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>24</v>
+      <c r="F7" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="8">
@@ -3901,14 +4105,14 @@
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="6">
         <v>9.2</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>27</v>
+      <c r="F8" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="9">
@@ -3921,14 +4125,14 @@
       <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>30</v>
+      <c r="E9" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="10">
@@ -3942,16 +4146,16 @@
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>31</v>
+        <v>64</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="11">
@@ -3964,11 +4168,11 @@
       <c r="C11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="6">
         <v>9.3</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>172</v>
+      <c r="F11" s="5" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="13">
@@ -3981,14 +4185,14 @@
       <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="6">
         <v>9.3</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>34</v>
+      <c r="F13" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="14">
@@ -4001,14 +4205,14 @@
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="6">
         <v>9.4</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>37</v>
+      <c r="F14" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15">
@@ -4021,14 +4225,14 @@
       <c r="C15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="6">
         <v>9.5</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>39</v>
+      <c r="F15" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="16">
@@ -4042,11 +4246,11 @@
         <v>6</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>42</v>
+      <c r="F16" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="17">
@@ -4060,8 +4264,8 @@
         <v>9</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="6" t="s">
-        <v>175</v>
+      <c r="F17" s="5" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="19">
@@ -4072,7 +4276,7 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20">
@@ -4085,14 +4289,14 @@
       <c r="C20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="6">
         <v>9.6</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>44</v>
+      <c r="F20" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -4105,14 +4309,14 @@
       <c r="C21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="6">
         <v>9.6</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>45</v>
+      <c r="F21" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -4125,14 +4329,14 @@
       <c r="C22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="6">
         <v>9.7</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>48</v>
+      <c r="F22" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -4145,11 +4349,11 @@
       <c r="C23" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="6">
         <v>9.8</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>179</v>
+      <c r="F23" s="5" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
@@ -4163,14 +4367,14 @@
       <c r="C25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="6">
         <v>9.8</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>49</v>
+      <c r="F25" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -4184,11 +4388,11 @@
         <v>15</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>52</v>
+      <c r="F26" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -4202,11 +4406,11 @@
         <v>19</v>
       </c>
       <c r="E27" s="1"/>
-      <c r="F27" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>54</v>
+      <c r="F27" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -4220,11 +4424,11 @@
         <v>6</v>
       </c>
       <c r="E28" s="1"/>
-      <c r="F28" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>57</v>
+      <c r="F28" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
@@ -4237,11 +4441,11 @@
       <c r="C29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>182</v>
+      <c r="E29" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1"/>
@@ -4255,14 +4459,14 @@
       <c r="C31" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="6">
         <v>10.1</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>59</v>
+      <c r="F31" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -4275,14 +4479,14 @@
       <c r="C32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="6">
         <v>10.2</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>61</v>
+      <c r="F32" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
@@ -4295,14 +4499,14 @@
       <c r="C33" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="6">
         <v>10.2</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>63</v>
+      <c r="F33" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
@@ -4316,16 +4520,16 @@
         <v>6</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="E34" s="5">
+        <v>213</v>
+      </c>
+      <c r="E34" s="6">
         <v>10.3</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>66</v>
+      <c r="F34" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -4339,8 +4543,8 @@
         <v>9</v>
       </c>
       <c r="E35" s="1"/>
-      <c r="F35" s="6" t="s">
-        <v>188</v>
+      <c r="F35" s="5" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1"/>
@@ -4354,14 +4558,14 @@
       <c r="C37" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E37" s="6">
         <v>10.4</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>68</v>
+      <c r="F37" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -4374,14 +4578,14 @@
       <c r="C38" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E38" s="5">
+      <c r="E38" s="6">
         <v>10.5</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>70</v>
+      <c r="F38" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -4394,14 +4598,14 @@
       <c r="C39" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="5">
+      <c r="E39" s="6">
         <v>10.6</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>72</v>
+      <c r="F39" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -4414,14 +4618,14 @@
       <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E40" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>74</v>
+      <c r="E40" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -4447,14 +4651,14 @@
       <c r="C43" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E43" s="5">
+      <c r="E43" s="6">
         <v>10.7</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>76</v>
+      <c r="F43" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -4468,11 +4672,11 @@
         <v>15</v>
       </c>
       <c r="E44" s="1"/>
-      <c r="F44" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>77</v>
+      <c r="F44" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -4486,11 +4690,11 @@
         <v>19</v>
       </c>
       <c r="E45" s="1"/>
-      <c r="F45" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>78</v>
+      <c r="F45" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -4504,11 +4708,11 @@
         <v>6</v>
       </c>
       <c r="E46" s="1"/>
-      <c r="F46" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>81</v>
+      <c r="F46" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -4522,8 +4726,8 @@
         <v>9</v>
       </c>
       <c r="E47" s="1"/>
-      <c r="F47" s="6" t="s">
-        <v>195</v>
+      <c r="F47" s="5" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>
@@ -4537,14 +4741,14 @@
       <c r="C49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E49" s="5">
+      <c r="E49" s="6">
         <v>11.1</v>
       </c>
-      <c r="F49" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>83</v>
+      <c r="F49" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -4557,14 +4761,14 @@
       <c r="C50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="5">
+      <c r="E50" s="6">
         <v>11.2</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>84</v>
+      <c r="F50" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -4577,14 +4781,14 @@
       <c r="C51" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E51" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>86</v>
+      <c r="E51" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
@@ -4595,15 +4799,15 @@
         <v>46471.0</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>199</v>
+        <v>238</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
       <c r="F52" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>89</v>
+        <v>236</v>
+      </c>
+      <c r="G52" s="11" t="s">
+        <v>239</v>
       </c>
       <c r="H52" s="10"/>
       <c r="I52" s="10"/>
@@ -4612,13 +4816,13 @@
     <row r="53" ht="15.75" customHeight="1"/>
     <row r="54" ht="15.75" customHeight="1">
       <c r="B54" s="1" t="s">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>202</v>
+        <v>242</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1"/>
@@ -4632,14 +4836,14 @@
       <c r="C56" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E56" s="5">
+      <c r="E56" s="6">
         <v>11.3</v>
       </c>
-      <c r="F56" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>90</v>
+      <c r="F56" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -4652,14 +4856,14 @@
       <c r="C57" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E57" s="5">
+      <c r="E57" s="6">
         <v>11.4</v>
       </c>
-      <c r="F57" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>92</v>
+      <c r="F57" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -4672,14 +4876,14 @@
       <c r="C58" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E58" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F58" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>95</v>
+      <c r="E58" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -4692,14 +4896,14 @@
       <c r="C59" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E59" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F59" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>97</v>
+      <c r="E59" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -4712,11 +4916,11 @@
       <c r="C60" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E60" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F60" s="6" t="s">
-        <v>205</v>
+      <c r="E60" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
@@ -4730,14 +4934,14 @@
       <c r="C62" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E62" s="5">
+      <c r="E62" s="6">
         <v>11.5</v>
       </c>
-      <c r="F62" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>99</v>
+      <c r="F62" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
@@ -4750,14 +4954,14 @@
       <c r="C63" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E63" s="5">
+      <c r="E63" s="6">
         <v>11.5</v>
       </c>
-      <c r="F63" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>101</v>
+      <c r="F63" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
@@ -4771,11 +4975,11 @@
         <v>19</v>
       </c>
       <c r="E64" s="1"/>
-      <c r="F64" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>103</v>
+      <c r="F64" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
@@ -4789,11 +4993,11 @@
         <v>6</v>
       </c>
       <c r="E65" s="1"/>
-      <c r="F65" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>104</v>
+      <c r="F65" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
@@ -4807,8 +5011,8 @@
         <v>9</v>
       </c>
       <c r="E66" s="1"/>
-      <c r="F66" s="6" t="s">
-        <v>208</v>
+      <c r="F66" s="5" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1"/>
@@ -4822,14 +5026,14 @@
       <c r="C68" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E68" s="5">
+      <c r="E68" s="6">
         <v>12.1</v>
       </c>
-      <c r="F68" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>106</v>
+      <c r="F68" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
@@ -4842,14 +5046,14 @@
       <c r="C69" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E69" s="5">
+      <c r="E69" s="6">
         <v>12.2</v>
       </c>
-      <c r="F69" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>109</v>
+      <c r="F69" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
@@ -4862,14 +5066,14 @@
       <c r="C70" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E70" s="5">
+      <c r="E70" s="6">
         <v>12.2</v>
       </c>
-      <c r="F70" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>111</v>
+      <c r="F70" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
@@ -4882,14 +5086,14 @@
       <c r="C71" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E71" s="5">
+      <c r="E71" s="6">
         <v>12.3</v>
       </c>
-      <c r="F71" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>113</v>
+      <c r="F71" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
@@ -4902,23 +5106,23 @@
       <c r="C72" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E72" s="5">
+      <c r="E72" s="6">
         <v>12.4</v>
       </c>
-      <c r="F72" s="6" t="s">
-        <v>212</v>
+      <c r="F72" s="5" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1">
       <c r="B74" s="1" t="s">
-        <v>213</v>
+        <v>265</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>214</v>
+        <v>266</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1"/>
@@ -4932,14 +5136,14 @@
       <c r="C76" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E76" s="5">
+      <c r="E76" s="6">
         <v>12.4</v>
       </c>
-      <c r="F76" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>114</v>
+      <c r="F76" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
@@ -4952,14 +5156,14 @@
       <c r="C77" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E77" s="5">
+      <c r="E77" s="6">
         <v>12.5</v>
       </c>
-      <c r="F77" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>119</v>
+      <c r="F77" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
@@ -4972,14 +5176,14 @@
       <c r="C78" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E78" s="5">
+      <c r="E78" s="6">
         <v>13.1</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>120</v>
+      <c r="F78" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="G78" s="6" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
@@ -4993,16 +5197,16 @@
         <v>6</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E79" s="5">
+        <v>64</v>
+      </c>
+      <c r="E79" s="6">
         <v>13.2</v>
       </c>
-      <c r="F79" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>122</v>
+      <c r="F79" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
@@ -5015,11 +5219,11 @@
       <c r="C80" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E80" s="5">
+      <c r="E80" s="6">
         <v>13.3</v>
       </c>
-      <c r="F80" s="6" t="s">
-        <v>219</v>
+      <c r="F80" s="5" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1"/>
@@ -5033,14 +5237,14 @@
       <c r="C82" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E82" s="5">
+      <c r="E82" s="6">
         <v>13.3</v>
       </c>
-      <c r="F82" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>123</v>
+      <c r="F82" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="G82" s="6" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
@@ -5053,14 +5257,14 @@
       <c r="C83" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E83" s="5">
+      <c r="E83" s="6">
         <v>13.4</v>
       </c>
-      <c r="F83" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>126</v>
+      <c r="F83" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="G83" s="6" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
@@ -5073,14 +5277,14 @@
       <c r="C84" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E84" s="5">
+      <c r="E84" s="6">
         <v>13.5</v>
       </c>
-      <c r="F84" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="G84" s="1" t="s">
-        <v>128</v>
+      <c r="F84" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="G84" s="6" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
@@ -5094,14 +5298,14 @@
         <v>6</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>222</v>
+        <v>281</v>
       </c>
       <c r="E85" s="1"/>
-      <c r="F85" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G85" s="1" t="s">
-        <v>130</v>
+      <c r="F85" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
@@ -5115,8 +5319,8 @@
         <v>9</v>
       </c>
       <c r="E86" s="1"/>
-      <c r="F86" s="6" t="s">
-        <v>223</v>
+      <c r="F86" s="5" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1"/>
@@ -5131,8 +5335,8 @@
         <v>11</v>
       </c>
       <c r="E88" s="1"/>
-      <c r="G88" s="1" t="s">
-        <v>133</v>
+      <c r="G88" s="6" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
@@ -5146,8 +5350,8 @@
         <v>15</v>
       </c>
       <c r="E89" s="1"/>
-      <c r="G89" s="1" t="s">
-        <v>135</v>
+      <c r="G89" s="6" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
@@ -5161,8 +5365,8 @@
         <v>19</v>
       </c>
       <c r="E90" s="1"/>
-      <c r="G90" s="1" t="s">
-        <v>137</v>
+      <c r="G90" s="6" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
@@ -5176,8 +5380,8 @@
         <v>6</v>
       </c>
       <c r="E91" s="1"/>
-      <c r="G91" s="1" t="s">
-        <v>139</v>
+      <c r="G91" s="6" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
@@ -5204,9 +5408,7 @@
         <v>11</v>
       </c>
       <c r="E94" s="1"/>
-      <c r="G94" s="1" t="s">
-        <v>140</v>
-      </c>
+      <c r="G94" s="1"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="1">
@@ -5219,9 +5421,7 @@
         <v>15</v>
       </c>
       <c r="E95" s="1"/>
-      <c r="G95" s="1" t="s">
-        <v>145</v>
-      </c>
+      <c r="G95" s="1"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="1">
@@ -5234,9 +5434,7 @@
         <v>19</v>
       </c>
       <c r="E96" s="1"/>
-      <c r="G96" s="1" t="s">
-        <v>146</v>
-      </c>
+      <c r="G96" s="1"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="1">
@@ -5248,9 +5446,7 @@
       <c r="C97" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G97" s="1" t="s">
-        <v>148</v>
-      </c>
+      <c r="G97" s="1"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="1">
@@ -5272,7 +5468,7 @@
         <v>11</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>224</v>
+        <v>288</v>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
@@ -5285,9 +5481,7 @@
       <c r="C101" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G101" s="1" t="s">
-        <v>149</v>
-      </c>
+      <c r="G101" s="1"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="1">
@@ -5299,9 +5493,7 @@
       <c r="C102" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G102" s="1" t="s">
-        <v>152</v>
-      </c>
+      <c r="G102" s="1"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="1">
@@ -5313,9 +5505,7 @@
       <c r="C103" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G103" s="1" t="s">
-        <v>153</v>
-      </c>
+      <c r="G103" s="1"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="7">
@@ -5325,10 +5515,10 @@
         <v>46542.0</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>225</v>
+        <v>289</v>
       </c>
       <c r="D104" s="7" t="s">
-        <v>226</v>
+        <v>290</v>
       </c>
       <c r="E104" s="7"/>
       <c r="F104" s="10"/>

</xml_diff>